<commit_message>
T03: fascia 22 x 225 / barge 22 x 250 sized from the 47 x 122 rafters at 45 deg (tails no longer below the soffit); price unchanged
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/T03/downloads/DG-T03 Turnkey BOQ.xlsx
+++ b/T03/downloads/DG-T03 Turnkey BOQ.xlsx
@@ -3815,7 +3815,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>uPVC fascia + vented soffit</t>
+          <t>uPVC fascia 22 x 225 + vented soffit</t>
         </is>
       </c>
       <c r="C9" s="8" t="n">
@@ -3858,7 +3858,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>uPVC barge boards 22 x 225</t>
+          <t>uPVC barge boards 22 x 250</t>
         </is>
       </c>
       <c r="C10" s="8" t="n">

</xml_diff>